<commit_message>
Add header block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/header/header.css
- blocks/header/header.js
- styles/styles.css
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/import-sustainability-topic.report.xlsx
- tools/importer/reports/import-what-we-do-topic.report.xlsx
- tools/importer/reports/index.report.json
- tools/importer/reports/sustainability.report.json
- tools/importer/reports/what-we-do.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="96">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","hero-marquee","columns-mosaic","carousel-article"]</t>
+    <t>["carousel-hero","hero-marquee","columns-mosaic","columns-feature","carousel-article"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-05-15T20:04:01.890Z</t>
+    <t>2026-05-15T20:42:01.285Z</t>
   </si>
   <si>
     <t>Chevron Corporation - Human Energy — Chevron</t>
@@ -70,7 +70,7 @@
     <t>investors</t>
   </si>
   <si>
-    <t>2026-05-14T22:08:04.337Z</t>
+    <t>2026-05-15T20:04:11.171Z</t>
   </si>
   <si>
     <t>Chevron Investors: Delivering Strong Results — Chevron</t>
@@ -82,13 +82,13 @@
     <t>sustainability.report.json</t>
   </si>
   <si>
-    <t>["hero-video","embed-map","cards-topic","carousel-article"]</t>
+    <t>["carousel-article"]</t>
   </si>
   <si>
     <t>sustainability</t>
   </si>
   <si>
-    <t>2026-05-14T20:00:15.122Z</t>
+    <t>2026-05-15T20:42:12.546Z</t>
   </si>
   <si>
     <t>Sustainability — Chevron.com — Chevron</t>
@@ -100,13 +100,10 @@
     <t>what-we-do.report.json</t>
   </si>
   <si>
-    <t>["hero-video","columns-mosaic","columns-mosaic","carousel-article"]</t>
-  </si>
-  <si>
     <t>what-we-do</t>
   </si>
   <si>
-    <t>2026-05-14T20:00:05.630Z</t>
+    <t>2026-05-15T20:42:22.333Z</t>
   </si>
   <si>
     <t>What We Do — Chevron</t>
@@ -792,7 +789,7 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
         <v>25</v>
@@ -809,285 +806,285 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>37</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>38</v>
-      </c>
-      <c r="H6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>42</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>43</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>45</v>
-      </c>
-      <c r="H7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>50</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>51</v>
-      </c>
-      <c r="H8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>54</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>56</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>57</v>
-      </c>
-      <c r="H9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
         <v>59</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>60</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>63</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>64</v>
-      </c>
-      <c r="H10" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
         <v>66</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>67</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
         <v>68</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>69</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>70</v>
-      </c>
-      <c r="H11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
         <v>72</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
         <v>74</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>75</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>76</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>77</v>
-      </c>
-      <c r="H12" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" t="s">
         <v>79</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>80</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>75</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>82</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>83</v>
-      </c>
-      <c r="H13" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" t="s">
         <v>85</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>86</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" t="s">
         <v>87</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>88</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>89</v>
-      </c>
-      <c r="H14" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
         <v>91</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>92</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" t="s">
         <v>93</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>94</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>95</v>
-      </c>
-      <c r="H15" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>